<commit_message>
update with NDC strategy, petroleum fix and more aggressive strategies
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20251030.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20251030.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tony/Documents/sisepuede_modeling/ssp_libya/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F691D2ED-4DD5-8342-860B-04653725490F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88695562-5C5B-904F-BEEA-358A98467D87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3120" yWindow="1640" windowWidth="28220" windowHeight="18140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="27040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,20 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">main!$A$1:$L$62</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">yaml!$A$1:$D$62</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1984,9 +1997,12 @@
         <v>0.5</v>
       </c>
       <c r="N2" s="18">
-        <v>1</v>
-      </c>
-      <c r="O2" s="11"/>
+        <v>2</v>
+      </c>
+      <c r="O2" s="11">
+        <f>K2*N2</f>
+        <v>0.9</v>
+      </c>
       <c r="P2" s="12"/>
       <c r="Q2" s="12"/>
     </row>
@@ -2021,7 +2037,10 @@
       </c>
       <c r="M3" s="18"/>
       <c r="N3" s="18"/>
-      <c r="O3" s="11"/>
+      <c r="O3" s="11">
+        <f t="shared" ref="O3:O8" si="0">K3*N3</f>
+        <v>0</v>
+      </c>
       <c r="P3" s="12"/>
       <c r="Q3" s="12"/>
     </row>
@@ -2056,7 +2075,10 @@
       </c>
       <c r="M4" s="18"/>
       <c r="N4" s="18"/>
-      <c r="O4" s="11"/>
+      <c r="O4" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="P4" s="12"/>
       <c r="Q4" s="12"/>
     </row>
@@ -2091,7 +2113,10 @@
       </c>
       <c r="M5" s="18"/>
       <c r="N5" s="18"/>
-      <c r="O5" s="11"/>
+      <c r="O5" s="11" t="e">
+        <f t="shared" si="0"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="P5" s="12"/>
       <c r="Q5" s="12"/>
     </row>
@@ -2130,7 +2155,10 @@
       </c>
       <c r="M6" s="18"/>
       <c r="N6" s="18"/>
-      <c r="O6" s="11"/>
+      <c r="O6" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="P6" s="12"/>
       <c r="Q6" s="12"/>
     </row>
@@ -2164,10 +2192,11 @@
         <v>12</v>
       </c>
       <c r="M7" s="18"/>
-      <c r="N7" s="18">
-        <v>1</v>
-      </c>
-      <c r="O7" s="11"/>
+      <c r="N7" s="18"/>
+      <c r="O7" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="P7" s="12"/>
       <c r="Q7" s="12"/>
     </row>
@@ -2205,12 +2234,15 @@
         <v>12</v>
       </c>
       <c r="M8" s="18">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="N8" s="18">
-        <v>1</v>
-      </c>
-      <c r="O8" s="11"/>
+        <v>2</v>
+      </c>
+      <c r="O8" s="11" t="e">
+        <f t="shared" si="0"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="P8" s="12"/>
       <c r="Q8" s="12"/>
     </row>
@@ -2249,9 +2281,12 @@
       </c>
       <c r="M9" s="18"/>
       <c r="N9" s="18">
-        <v>1</v>
-      </c>
-      <c r="O9" s="11"/>
+        <v>1.05</v>
+      </c>
+      <c r="O9" s="11">
+        <f>K9*N9</f>
+        <v>0.99749999999999994</v>
+      </c>
       <c r="P9" s="12"/>
       <c r="Q9" s="12"/>
     </row>
@@ -2289,12 +2324,15 @@
         <v>12</v>
       </c>
       <c r="M10" s="18">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="N10" s="18">
-        <v>1</v>
-      </c>
-      <c r="O10" s="11"/>
+        <v>1.05</v>
+      </c>
+      <c r="O10" s="11">
+        <f t="shared" ref="O10:O62" si="1">K10*N10</f>
+        <v>0.99749999999999994</v>
+      </c>
       <c r="P10" s="12"/>
       <c r="Q10" s="12"/>
     </row>
@@ -2327,11 +2365,16 @@
       <c r="L11" s="17">
         <v>12</v>
       </c>
-      <c r="M11" s="18"/>
+      <c r="M11" s="18">
+        <v>0.1</v>
+      </c>
       <c r="N11" s="18">
-        <v>1</v>
-      </c>
-      <c r="O11" s="11"/>
+        <v>1.25</v>
+      </c>
+      <c r="O11" s="11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
       <c r="P11" s="12"/>
       <c r="Q11" s="12"/>
     </row>
@@ -2364,11 +2407,16 @@
       <c r="L12" s="17">
         <v>12</v>
       </c>
-      <c r="M12" s="18"/>
+      <c r="M12" s="18">
+        <v>0.1</v>
+      </c>
       <c r="N12" s="18">
-        <v>1</v>
-      </c>
-      <c r="O12" s="11"/>
+        <v>1.25</v>
+      </c>
+      <c r="O12" s="11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
       <c r="P12" s="12"/>
       <c r="Q12" s="12"/>
     </row>
@@ -2406,12 +2454,15 @@
         <v>12</v>
       </c>
       <c r="M13" s="18">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="N13" s="18">
-        <v>1</v>
-      </c>
-      <c r="O13" s="11"/>
+        <v>2.5</v>
+      </c>
+      <c r="O13" s="11">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
       <c r="P13" s="12"/>
       <c r="Q13" s="12"/>
     </row>
@@ -2449,12 +2500,15 @@
         <v>12</v>
       </c>
       <c r="M14" s="18">
+        <v>1</v>
+      </c>
+      <c r="N14" s="18">
+        <v>2</v>
+      </c>
+      <c r="O14" s="11">
+        <f t="shared" si="1"/>
         <v>0.8</v>
       </c>
-      <c r="N14" s="18">
-        <v>1</v>
-      </c>
-      <c r="O14" s="11"/>
       <c r="P14" s="12"/>
       <c r="Q14" s="12"/>
     </row>
@@ -2491,7 +2545,10 @@
       <c r="N15" s="18">
         <v>1</v>
       </c>
-      <c r="O15" s="11"/>
+      <c r="O15" s="11" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="P15" s="12"/>
       <c r="Q15" s="12"/>
     </row>
@@ -2528,13 +2585,14 @@
       <c r="L16" s="17">
         <v>12</v>
       </c>
-      <c r="M16" s="18">
-        <v>1</v>
-      </c>
+      <c r="M16" s="18"/>
       <c r="N16" s="18">
-        <v>1</v>
-      </c>
-      <c r="O16" s="11"/>
+        <v>1.8</v>
+      </c>
+      <c r="O16" s="11">
+        <f t="shared" si="1"/>
+        <v>0.9</v>
+      </c>
       <c r="P16" s="12"/>
       <c r="Q16" s="12"/>
     </row>
@@ -2573,9 +2631,12 @@
       </c>
       <c r="M17" s="18"/>
       <c r="N17" s="18">
-        <v>1</v>
-      </c>
-      <c r="O17" s="11"/>
+        <v>1.7</v>
+      </c>
+      <c r="O17" s="11">
+        <f t="shared" si="1"/>
+        <v>0.51</v>
+      </c>
       <c r="P17" s="12"/>
       <c r="Q17" s="12"/>
     </row>
@@ -2616,9 +2677,12 @@
         <v>1</v>
       </c>
       <c r="N18" s="18">
-        <v>1</v>
-      </c>
-      <c r="O18" s="11"/>
+        <v>2</v>
+      </c>
+      <c r="O18" s="11">
+        <f t="shared" si="1"/>
+        <v>0.2</v>
+      </c>
       <c r="P18" s="12"/>
       <c r="Q18" s="12"/>
     </row>
@@ -2651,13 +2715,14 @@
       <c r="L19" s="17">
         <v>12</v>
       </c>
-      <c r="M19" s="18">
-        <v>1</v>
-      </c>
+      <c r="M19" s="18"/>
       <c r="N19" s="18">
-        <v>1</v>
-      </c>
-      <c r="O19" s="11"/>
+        <v>2</v>
+      </c>
+      <c r="O19" s="11">
+        <f t="shared" si="1"/>
+        <v>0.2</v>
+      </c>
       <c r="P19" s="12"/>
       <c r="Q19" s="12"/>
     </row>
@@ -2694,9 +2759,12 @@
         <v>1</v>
       </c>
       <c r="N20" s="18">
-        <v>1</v>
-      </c>
-      <c r="O20" s="11"/>
+        <v>2</v>
+      </c>
+      <c r="O20" s="11">
+        <f t="shared" si="1"/>
+        <v>0.2</v>
+      </c>
       <c r="P20" s="12"/>
       <c r="Q20" s="12"/>
     </row>
@@ -2733,9 +2801,12 @@
         <v>1</v>
       </c>
       <c r="N21" s="18">
-        <v>1</v>
-      </c>
-      <c r="O21" s="11"/>
+        <v>2</v>
+      </c>
+      <c r="O21" s="11">
+        <f t="shared" si="1"/>
+        <v>0.2</v>
+      </c>
       <c r="P21" s="12"/>
       <c r="Q21" s="12"/>
     </row>
@@ -2773,10 +2844,11 @@
         <v>12</v>
       </c>
       <c r="M22" s="18"/>
-      <c r="N22" s="18">
-        <v>1</v>
-      </c>
-      <c r="O22" s="11"/>
+      <c r="N22" s="18"/>
+      <c r="O22" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="P22" s="12"/>
       <c r="Q22" s="12"/>
     </row>
@@ -2814,10 +2886,11 @@
         <v>12</v>
       </c>
       <c r="M23" s="18"/>
-      <c r="N23" s="18">
-        <v>1</v>
-      </c>
-      <c r="O23" s="11"/>
+      <c r="N23" s="18"/>
+      <c r="O23" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="P23" s="12"/>
       <c r="Q23" s="12"/>
     </row>
@@ -2855,10 +2928,11 @@
         <v>12</v>
       </c>
       <c r="M24" s="18"/>
-      <c r="N24" s="18">
-        <v>1</v>
-      </c>
-      <c r="O24" s="11"/>
+      <c r="N24" s="18"/>
+      <c r="O24" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="P24" s="12"/>
       <c r="Q24" s="12"/>
     </row>
@@ -2896,10 +2970,11 @@
         <v>12</v>
       </c>
       <c r="M25" s="18"/>
-      <c r="N25" s="18">
-        <v>1</v>
-      </c>
-      <c r="O25" s="11"/>
+      <c r="N25" s="18"/>
+      <c r="O25" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="P25" s="12"/>
       <c r="Q25" s="12"/>
     </row>
@@ -2938,7 +3013,10 @@
       <c r="N26" s="18">
         <v>1</v>
       </c>
-      <c r="O26" s="29"/>
+      <c r="O26" s="11">
+        <f t="shared" si="1"/>
+        <v>0.9</v>
+      </c>
       <c r="P26" s="12"/>
       <c r="Q26" s="30"/>
     </row>
@@ -2977,7 +3055,10 @@
       <c r="N27" s="18">
         <v>1</v>
       </c>
-      <c r="O27" s="11"/>
+      <c r="O27" s="11" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="P27" s="12"/>
       <c r="Q27" s="12"/>
     </row>
@@ -3016,7 +3097,10 @@
       <c r="N28" s="18">
         <v>1</v>
       </c>
-      <c r="O28" s="11"/>
+      <c r="O28" s="11" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="P28" s="12"/>
       <c r="Q28" s="12"/>
     </row>
@@ -3055,7 +3139,10 @@
       <c r="N29" s="18">
         <v>1</v>
       </c>
-      <c r="O29" s="11"/>
+      <c r="O29" s="11" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="P29" s="12"/>
       <c r="Q29" s="12"/>
     </row>
@@ -3094,7 +3181,10 @@
       <c r="N30" s="18">
         <v>1</v>
       </c>
-      <c r="O30" s="11"/>
+      <c r="O30" s="11" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="P30" s="12"/>
       <c r="Q30" s="12"/>
     </row>
@@ -3127,11 +3217,16 @@
       <c r="L31" s="17">
         <v>12</v>
       </c>
-      <c r="M31" s="18"/>
+      <c r="M31" s="18">
+        <v>1</v>
+      </c>
       <c r="N31" s="18">
-        <v>1</v>
-      </c>
-      <c r="O31" s="11"/>
+        <v>1.5</v>
+      </c>
+      <c r="O31" s="11">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
       <c r="P31" s="12"/>
       <c r="Q31" s="12"/>
     </row>
@@ -3169,12 +3264,15 @@
         <v>12</v>
       </c>
       <c r="M32" s="18">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="N32" s="18">
-        <v>1</v>
-      </c>
-      <c r="O32" s="29"/>
+        <v>2</v>
+      </c>
+      <c r="O32" s="11">
+        <f t="shared" si="1"/>
+        <v>0.6</v>
+      </c>
       <c r="P32" s="18"/>
       <c r="Q32" s="31"/>
     </row>
@@ -3207,11 +3305,16 @@
       <c r="L33" s="17">
         <v>12</v>
       </c>
-      <c r="M33" s="18"/>
+      <c r="M33" s="18">
+        <v>1</v>
+      </c>
       <c r="N33" s="18">
-        <v>1</v>
-      </c>
-      <c r="O33" s="11"/>
+        <v>1.5</v>
+      </c>
+      <c r="O33" s="11">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
       <c r="P33" s="12"/>
       <c r="Q33" s="12"/>
     </row>
@@ -3244,11 +3347,16 @@
       <c r="L34" s="17">
         <v>12</v>
       </c>
-      <c r="M34" s="18"/>
+      <c r="M34" s="18">
+        <v>1</v>
+      </c>
       <c r="N34" s="18">
-        <v>1</v>
-      </c>
-      <c r="O34" s="11"/>
+        <v>1.5</v>
+      </c>
+      <c r="O34" s="11">
+        <f t="shared" si="1"/>
+        <v>1.35</v>
+      </c>
       <c r="P34" s="12"/>
       <c r="Q34" s="12"/>
     </row>
@@ -3282,12 +3390,15 @@
         <v>12</v>
       </c>
       <c r="M35" s="18">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="N35" s="18">
-        <v>1</v>
-      </c>
-      <c r="O35" s="11"/>
+        <v>1.5</v>
+      </c>
+      <c r="O35" s="11">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
       <c r="P35" s="12"/>
       <c r="Q35" s="12"/>
     </row>
@@ -3321,12 +3432,15 @@
         <v>12</v>
       </c>
       <c r="M36" s="18">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="N36" s="18">
-        <v>1</v>
-      </c>
-      <c r="O36" s="11"/>
+        <v>1.5</v>
+      </c>
+      <c r="O36" s="11">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
       <c r="P36" s="12"/>
       <c r="Q36" s="12"/>
     </row>
@@ -3360,12 +3474,15 @@
         <v>12</v>
       </c>
       <c r="M37" s="18">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="N37" s="18">
         <v>1</v>
       </c>
-      <c r="O37" s="11"/>
+      <c r="O37" s="11">
+        <f t="shared" si="1"/>
+        <v>0.95</v>
+      </c>
       <c r="P37" s="12"/>
       <c r="Q37" s="12"/>
     </row>
@@ -3399,10 +3516,11 @@
         <v>12</v>
       </c>
       <c r="M38" s="18"/>
-      <c r="N38" s="18">
-        <v>1</v>
-      </c>
-      <c r="O38" s="11"/>
+      <c r="N38" s="18"/>
+      <c r="O38" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="P38" s="12"/>
       <c r="Q38" s="12"/>
     </row>
@@ -3436,10 +3554,11 @@
         <v>12</v>
       </c>
       <c r="M39" s="18"/>
-      <c r="N39" s="18">
-        <v>1</v>
-      </c>
-      <c r="O39" s="11"/>
+      <c r="N39" s="18"/>
+      <c r="O39" s="11">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
       <c r="P39" s="12"/>
       <c r="Q39" s="12"/>
     </row>
@@ -3477,12 +3596,15 @@
         <v>12</v>
       </c>
       <c r="M40" s="18">
-        <v>0.8</v>
+        <v>2</v>
       </c>
       <c r="N40" s="18">
-        <v>1</v>
-      </c>
-      <c r="O40" s="11"/>
+        <v>3</v>
+      </c>
+      <c r="O40" s="11">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
       <c r="P40" s="12"/>
       <c r="Q40" s="12"/>
     </row>
@@ -3519,11 +3641,16 @@
       <c r="L41" s="17">
         <v>12</v>
       </c>
-      <c r="M41" s="18"/>
+      <c r="M41" s="18">
+        <v>2</v>
+      </c>
       <c r="N41" s="18">
-        <v>1</v>
-      </c>
-      <c r="O41" s="11"/>
+        <v>3</v>
+      </c>
+      <c r="O41" s="11">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
       <c r="P41" s="12"/>
       <c r="Q41" s="12"/>
     </row>
@@ -3560,11 +3687,16 @@
       <c r="L42" s="17">
         <v>12</v>
       </c>
-      <c r="M42" s="18"/>
+      <c r="M42" s="18">
+        <v>2</v>
+      </c>
       <c r="N42" s="18">
-        <v>1</v>
-      </c>
-      <c r="O42" s="11"/>
+        <v>3</v>
+      </c>
+      <c r="O42" s="11">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
       <c r="P42" s="12"/>
       <c r="Q42" s="12"/>
     </row>
@@ -3598,12 +3730,15 @@
         <v>12</v>
       </c>
       <c r="M43" s="18">
-        <v>0.8</v>
+        <v>2</v>
       </c>
       <c r="N43" s="18">
-        <v>1</v>
-      </c>
-      <c r="O43" s="11"/>
+        <v>3</v>
+      </c>
+      <c r="O43" s="11">
+        <f t="shared" si="1"/>
+        <v>0.75</v>
+      </c>
       <c r="P43" s="12"/>
       <c r="Q43" s="12"/>
     </row>
@@ -3637,12 +3772,15 @@
         <v>12</v>
       </c>
       <c r="M44" s="18">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="N44" s="18">
-        <v>1</v>
-      </c>
-      <c r="O44" s="11"/>
+        <v>1.5</v>
+      </c>
+      <c r="O44" s="11">
+        <f t="shared" si="1"/>
+        <v>1.0499999999999998</v>
+      </c>
       <c r="P44" s="12"/>
       <c r="Q44" s="12"/>
     </row>
@@ -3680,12 +3818,15 @@
         <v>12</v>
       </c>
       <c r="M45" s="18">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="N45" s="18">
-        <v>1</v>
-      </c>
-      <c r="O45" s="11"/>
+        <v>2</v>
+      </c>
+      <c r="O45" s="11">
+        <f t="shared" si="1"/>
+        <v>1.4</v>
+      </c>
       <c r="P45" s="12"/>
       <c r="Q45" s="12"/>
     </row>
@@ -3723,12 +3864,15 @@
         <v>12</v>
       </c>
       <c r="M46" s="18">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="N46" s="18">
-        <v>1</v>
-      </c>
-      <c r="O46" s="11"/>
+        <v>2</v>
+      </c>
+      <c r="O46" s="11">
+        <f t="shared" si="1"/>
+        <v>1.4</v>
+      </c>
       <c r="P46" s="12"/>
       <c r="Q46" s="12"/>
     </row>
@@ -3761,11 +3905,16 @@
       <c r="L47" s="17">
         <v>12</v>
       </c>
-      <c r="M47" s="18"/>
+      <c r="M47" s="18">
+        <v>1</v>
+      </c>
       <c r="N47" s="18">
-        <v>1</v>
-      </c>
-      <c r="O47" s="11"/>
+        <v>2</v>
+      </c>
+      <c r="O47" s="11">
+        <f t="shared" si="1"/>
+        <v>0.5</v>
+      </c>
       <c r="P47" s="12"/>
       <c r="Q47" s="12"/>
     </row>
@@ -3803,12 +3952,15 @@
         <v>12</v>
       </c>
       <c r="M48" s="18">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="N48" s="18">
-        <v>1</v>
-      </c>
-      <c r="O48" s="11"/>
+        <v>2</v>
+      </c>
+      <c r="O48" s="11">
+        <f t="shared" si="1"/>
+        <v>0.4</v>
+      </c>
       <c r="P48" s="12"/>
       <c r="Q48" s="12"/>
     </row>
@@ -3846,12 +3998,15 @@
         <v>12</v>
       </c>
       <c r="M49" s="18">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="N49" s="18">
-        <v>1</v>
-      </c>
-      <c r="O49" s="11"/>
+        <v>2</v>
+      </c>
+      <c r="O49" s="11">
+        <f t="shared" si="1"/>
+        <v>0.6</v>
+      </c>
       <c r="P49" s="12"/>
       <c r="Q49" s="12"/>
     </row>
@@ -3889,12 +4044,15 @@
         <v>12</v>
       </c>
       <c r="M50" s="18">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="N50" s="18">
         <v>1</v>
       </c>
-      <c r="O50" s="11"/>
+      <c r="O50" s="11" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="P50" s="12"/>
       <c r="Q50" s="12"/>
     </row>
@@ -3927,11 +4085,16 @@
       <c r="L51" s="17">
         <v>12</v>
       </c>
-      <c r="M51" s="18"/>
+      <c r="M51" s="18">
+        <v>1</v>
+      </c>
       <c r="N51" s="18">
         <v>1</v>
       </c>
-      <c r="O51" s="11"/>
+      <c r="O51" s="11">
+        <f t="shared" si="1"/>
+        <v>0.85</v>
+      </c>
       <c r="P51" s="12"/>
       <c r="Q51" s="12"/>
     </row>
@@ -3968,11 +4131,16 @@
       <c r="L52" s="17">
         <v>12</v>
       </c>
-      <c r="M52" s="18"/>
+      <c r="M52" s="18">
+        <v>1</v>
+      </c>
       <c r="N52" s="18">
         <v>1</v>
       </c>
-      <c r="O52" s="11"/>
+      <c r="O52" s="11">
+        <f t="shared" si="1"/>
+        <v>0.9</v>
+      </c>
       <c r="P52" s="12"/>
       <c r="Q52" s="12"/>
     </row>
@@ -4009,11 +4177,16 @@
       <c r="L53" s="17">
         <v>12</v>
       </c>
-      <c r="M53" s="18"/>
+      <c r="M53" s="18">
+        <v>1</v>
+      </c>
       <c r="N53" s="18">
         <v>1</v>
       </c>
-      <c r="O53" s="11"/>
+      <c r="O53" s="11" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="P53" s="12"/>
       <c r="Q53" s="12"/>
     </row>
@@ -4050,11 +4223,16 @@
       <c r="L54" s="17">
         <v>12</v>
       </c>
-      <c r="M54" s="18"/>
+      <c r="M54" s="18">
+        <v>1</v>
+      </c>
       <c r="N54" s="18">
         <v>1</v>
       </c>
-      <c r="O54" s="11"/>
+      <c r="O54" s="11" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="P54" s="12"/>
       <c r="Q54" s="12"/>
     </row>
@@ -4091,11 +4269,16 @@
       <c r="L55" s="17">
         <v>12</v>
       </c>
-      <c r="M55" s="18"/>
+      <c r="M55" s="18">
+        <v>1</v>
+      </c>
       <c r="N55" s="18">
         <v>1</v>
       </c>
-      <c r="O55" s="11"/>
+      <c r="O55" s="11" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="P55" s="12"/>
       <c r="Q55" s="12"/>
     </row>
@@ -4132,11 +4315,16 @@
       <c r="L56" s="17">
         <v>12</v>
       </c>
-      <c r="M56" s="18"/>
+      <c r="M56" s="18">
+        <v>1</v>
+      </c>
       <c r="N56" s="18">
         <v>1</v>
       </c>
-      <c r="O56" s="11"/>
+      <c r="O56" s="11">
+        <f t="shared" si="1"/>
+        <v>0.3</v>
+      </c>
       <c r="P56" s="12"/>
       <c r="Q56" s="12"/>
     </row>
@@ -4171,7 +4359,10 @@
       </c>
       <c r="M57" s="18"/>
       <c r="N57" s="18"/>
-      <c r="O57" s="11"/>
+      <c r="O57" s="11" t="e">
+        <f t="shared" si="1"/>
+        <v>#VALUE!</v>
+      </c>
       <c r="P57" s="12"/>
       <c r="Q57" s="12"/>
     </row>
@@ -4208,11 +4399,16 @@
       <c r="L58" s="17">
         <v>12</v>
       </c>
-      <c r="M58" s="18"/>
+      <c r="M58" s="18">
+        <v>1</v>
+      </c>
       <c r="N58" s="18">
         <v>1</v>
       </c>
-      <c r="O58" s="11"/>
+      <c r="O58" s="11">
+        <f t="shared" si="1"/>
+        <v>0.85</v>
+      </c>
       <c r="P58" s="12"/>
       <c r="Q58" s="12"/>
     </row>
@@ -4245,11 +4441,16 @@
       <c r="L59" s="17">
         <v>12</v>
       </c>
-      <c r="M59" s="18"/>
+      <c r="M59" s="18">
+        <v>1</v>
+      </c>
       <c r="N59" s="18">
         <v>1</v>
       </c>
-      <c r="O59" s="11"/>
+      <c r="O59" s="11">
+        <f t="shared" si="1"/>
+        <v>0.85</v>
+      </c>
       <c r="P59" s="12"/>
       <c r="Q59" s="12"/>
     </row>
@@ -4282,11 +4483,16 @@
       <c r="L60" s="17">
         <v>12</v>
       </c>
-      <c r="M60" s="18"/>
+      <c r="M60" s="18">
+        <v>1</v>
+      </c>
       <c r="N60" s="18">
         <v>1</v>
       </c>
-      <c r="O60" s="11"/>
+      <c r="O60" s="11">
+        <f t="shared" si="1"/>
+        <v>0.85</v>
+      </c>
       <c r="P60" s="12"/>
       <c r="Q60" s="12"/>
     </row>
@@ -4329,7 +4535,10 @@
       <c r="N61" s="18">
         <v>1</v>
       </c>
-      <c r="O61" s="11"/>
+      <c r="O61" s="11">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
       <c r="P61" s="12"/>
       <c r="Q61" s="12"/>
     </row>
@@ -4372,7 +4581,10 @@
       <c r="N62" s="18">
         <v>1</v>
       </c>
-      <c r="O62" s="11"/>
+      <c r="O62" s="11">
+        <f t="shared" si="1"/>
+        <v>0.95</v>
+      </c>
       <c r="P62" s="12"/>
       <c r="Q62" s="12"/>
     </row>

</xml_diff>

<commit_message>
update notebooks and postprocessing files for nov 4th update
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20251030.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20251030.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tony/Documents/sisepuede_modeling/ssp_libya/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88695562-5C5B-904F-BEEA-358A98467D87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9A59812-152F-4241-9334-2CC9BF826C0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="68800" windowHeight="27040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20400" yWindow="2580" windowWidth="15360" windowHeight="17740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="412">
   <si>
     <t>subsector</t>
   </si>
@@ -1308,6 +1308,18 @@
   </si>
   <si>
     <t>strategy_NDC</t>
+  </si>
+  <si>
+    <t>TX:ENFU:ADJ_EXPORTS</t>
+  </si>
+  <si>
+    <t>ENFU</t>
+  </si>
+  <si>
+    <t>Increase fuel exports</t>
+  </si>
+  <si>
+    <t>transformation_enfu_adj_exports.yaml</t>
   </si>
 </sst>
 </file>
@@ -1377,7 +1389,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -1465,11 +1477,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1567,9 +1607,6 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -1596,6 +1633,60 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1902,19 +1993,21 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:Q65"/>
+  <dimension ref="A1:Q64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="13.1640625" style="37" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.5" style="37" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.5" style="37" bestFit="1" customWidth="1"/>
-    <col min="5" max="10" width="13" style="37" hidden="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="31.5" style="38" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="19.83203125" style="39" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="20.5" style="40" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.5" style="41" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.5" style="40" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.5" style="42" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="13.1640625" style="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.5" style="36" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.5" style="36" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="49.83203125" style="36" customWidth="1"/>
+    <col min="6" max="6" width="88.33203125" style="36" hidden="1" customWidth="1"/>
+    <col min="7" max="10" width="13" style="36" hidden="1" customWidth="1"/>
+    <col min="11" max="11" width="31.5" style="37" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.83203125" style="38" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="20.5" style="39" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.5" style="40" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.5" style="39" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.5" style="41" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" s="4" customFormat="1" ht="65" customHeight="1" x14ac:dyDescent="0.2">
@@ -1993,15 +2086,11 @@
       <c r="L2" s="17">
         <v>12</v>
       </c>
-      <c r="M2" s="18">
-        <v>0.5</v>
-      </c>
-      <c r="N2" s="18">
-        <v>2</v>
-      </c>
+      <c r="M2" s="18"/>
+      <c r="N2" s="18"/>
       <c r="O2" s="11">
         <f>K2*N2</f>
-        <v>0.9</v>
+        <v>0</v>
       </c>
       <c r="P2" s="12"/>
       <c r="Q2" s="12"/>
@@ -2233,12 +2322,8 @@
       <c r="L8" s="17">
         <v>12</v>
       </c>
-      <c r="M8" s="18">
-        <v>1</v>
-      </c>
-      <c r="N8" s="18">
-        <v>2</v>
-      </c>
+      <c r="M8" s="18"/>
+      <c r="N8" s="18"/>
       <c r="O8" s="11" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
@@ -2280,12 +2365,10 @@
         <v>12</v>
       </c>
       <c r="M9" s="18"/>
-      <c r="N9" s="18">
-        <v>1.05</v>
-      </c>
+      <c r="N9" s="18"/>
       <c r="O9" s="11">
         <f>K9*N9</f>
-        <v>0.99749999999999994</v>
+        <v>0</v>
       </c>
       <c r="P9" s="12"/>
       <c r="Q9" s="12"/>
@@ -2324,14 +2407,14 @@
         <v>12</v>
       </c>
       <c r="M10" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="N10" s="18">
         <v>1</v>
       </c>
-      <c r="N10" s="18">
-        <v>1.05</v>
-      </c>
       <c r="O10" s="11">
-        <f t="shared" ref="O10:O62" si="1">K10*N10</f>
-        <v>0.99749999999999994</v>
+        <f t="shared" ref="O10:O63" si="1">K10*N10</f>
+        <v>0.95</v>
       </c>
       <c r="P10" s="12"/>
       <c r="Q10" s="12"/>
@@ -2366,14 +2449,14 @@
         <v>12</v>
       </c>
       <c r="M11" s="18">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="N11" s="18">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="O11" s="11">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="P11" s="12"/>
       <c r="Q11" s="12"/>
@@ -2408,14 +2491,14 @@
         <v>12</v>
       </c>
       <c r="M12" s="18">
-        <v>0.1</v>
+        <v>0.5</v>
       </c>
       <c r="N12" s="18">
-        <v>1.25</v>
+        <v>1</v>
       </c>
       <c r="O12" s="11">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="P12" s="12"/>
       <c r="Q12" s="12"/>
@@ -2453,15 +2536,11 @@
       <c r="L13" s="17">
         <v>12</v>
       </c>
-      <c r="M13" s="18">
-        <v>1</v>
-      </c>
-      <c r="N13" s="18">
-        <v>2.5</v>
-      </c>
+      <c r="M13" s="18"/>
+      <c r="N13" s="18"/>
       <c r="O13" s="11">
         <f t="shared" si="1"/>
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="P13" s="12"/>
       <c r="Q13" s="12"/>
@@ -2499,15 +2578,11 @@
       <c r="L14" s="17">
         <v>12</v>
       </c>
-      <c r="M14" s="18">
-        <v>1</v>
-      </c>
-      <c r="N14" s="18">
-        <v>2</v>
-      </c>
+      <c r="M14" s="18"/>
+      <c r="N14" s="18"/>
       <c r="O14" s="11">
         <f t="shared" si="1"/>
-        <v>0.8</v>
+        <v>0</v>
       </c>
       <c r="P14" s="12"/>
       <c r="Q14" s="12"/>
@@ -2542,9 +2617,7 @@
         <v>12</v>
       </c>
       <c r="M15" s="18"/>
-      <c r="N15" s="18">
-        <v>1</v>
-      </c>
+      <c r="N15" s="18"/>
       <c r="O15" s="11" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
@@ -2673,9 +2746,7 @@
       <c r="L18" s="17">
         <v>12</v>
       </c>
-      <c r="M18" s="18">
-        <v>1</v>
-      </c>
+      <c r="M18" s="18"/>
       <c r="N18" s="18">
         <v>2</v>
       </c>
@@ -2755,9 +2826,7 @@
       <c r="L20" s="17">
         <v>12</v>
       </c>
-      <c r="M20" s="18">
-        <v>1</v>
-      </c>
+      <c r="M20" s="18"/>
       <c r="N20" s="18">
         <v>2</v>
       </c>
@@ -2797,9 +2866,7 @@
       <c r="L21" s="17">
         <v>12</v>
       </c>
-      <c r="M21" s="18">
-        <v>1</v>
-      </c>
+      <c r="M21" s="18"/>
       <c r="N21" s="18">
         <v>2</v>
       </c>
@@ -3305,9 +3372,7 @@
       <c r="L33" s="17">
         <v>12</v>
       </c>
-      <c r="M33" s="18">
-        <v>1</v>
-      </c>
+      <c r="M33" s="18"/>
       <c r="N33" s="18">
         <v>1.5</v>
       </c>
@@ -3347,9 +3412,7 @@
       <c r="L34" s="17">
         <v>12</v>
       </c>
-      <c r="M34" s="18">
-        <v>1</v>
-      </c>
+      <c r="M34" s="18"/>
       <c r="N34" s="18">
         <v>1.5</v>
       </c>
@@ -3390,14 +3453,14 @@
         <v>12</v>
       </c>
       <c r="M35" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="N35" s="18">
         <v>1</v>
-      </c>
-      <c r="N35" s="18">
-        <v>1.5</v>
       </c>
       <c r="O35" s="11">
         <f t="shared" si="1"/>
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="P35" s="12"/>
       <c r="Q35" s="12"/>
@@ -3431,15 +3494,11 @@
       <c r="L36" s="17">
         <v>12</v>
       </c>
-      <c r="M36" s="18">
-        <v>1</v>
-      </c>
-      <c r="N36" s="18">
-        <v>1.5</v>
-      </c>
+      <c r="M36" s="18"/>
+      <c r="N36" s="18"/>
       <c r="O36" s="11">
         <f t="shared" si="1"/>
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="P36" s="12"/>
       <c r="Q36" s="12"/>
@@ -3474,7 +3533,7 @@
         <v>12</v>
       </c>
       <c r="M37" s="18">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="N37" s="18">
         <v>1</v>
@@ -3595,9 +3654,7 @@
       <c r="L40" s="17">
         <v>12</v>
       </c>
-      <c r="M40" s="18">
-        <v>2</v>
-      </c>
+      <c r="M40" s="18"/>
       <c r="N40" s="18">
         <v>3</v>
       </c>
@@ -3641,15 +3698,11 @@
       <c r="L41" s="17">
         <v>12</v>
       </c>
-      <c r="M41" s="18">
-        <v>2</v>
-      </c>
-      <c r="N41" s="18">
-        <v>3</v>
-      </c>
+      <c r="M41" s="18"/>
+      <c r="N41" s="18"/>
       <c r="O41" s="11">
         <f t="shared" si="1"/>
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="P41" s="12"/>
       <c r="Q41" s="12"/>
@@ -3687,15 +3740,11 @@
       <c r="L42" s="17">
         <v>12</v>
       </c>
-      <c r="M42" s="18">
-        <v>2</v>
-      </c>
-      <c r="N42" s="18">
-        <v>3</v>
-      </c>
+      <c r="M42" s="18"/>
+      <c r="N42" s="18"/>
       <c r="O42" s="11">
         <f t="shared" si="1"/>
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="P42" s="12"/>
       <c r="Q42" s="12"/>
@@ -3729,9 +3778,7 @@
       <c r="L43" s="17">
         <v>12</v>
       </c>
-      <c r="M43" s="18">
-        <v>2</v>
-      </c>
+      <c r="M43" s="18"/>
       <c r="N43" s="18">
         <v>3</v>
       </c>
@@ -3772,14 +3819,14 @@
         <v>12</v>
       </c>
       <c r="M44" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="N44" s="18">
         <v>1</v>
-      </c>
-      <c r="N44" s="18">
-        <v>1.5</v>
       </c>
       <c r="O44" s="11">
         <f t="shared" si="1"/>
-        <v>1.0499999999999998</v>
+        <v>0.7</v>
       </c>
       <c r="P44" s="12"/>
       <c r="Q44" s="12"/>
@@ -3818,14 +3865,14 @@
         <v>12</v>
       </c>
       <c r="M45" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="N45" s="18">
         <v>1</v>
-      </c>
-      <c r="N45" s="18">
-        <v>2</v>
       </c>
       <c r="O45" s="11">
         <f t="shared" si="1"/>
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="P45" s="12"/>
       <c r="Q45" s="12"/>
@@ -3864,14 +3911,14 @@
         <v>12</v>
       </c>
       <c r="M46" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="N46" s="18">
         <v>1</v>
-      </c>
-      <c r="N46" s="18">
-        <v>2</v>
       </c>
       <c r="O46" s="11">
         <f t="shared" si="1"/>
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="P46" s="12"/>
       <c r="Q46" s="12"/>
@@ -3906,14 +3953,14 @@
         <v>12</v>
       </c>
       <c r="M47" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="N47" s="18">
         <v>1</v>
-      </c>
-      <c r="N47" s="18">
-        <v>2</v>
       </c>
       <c r="O47" s="11">
         <f t="shared" si="1"/>
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="P47" s="12"/>
       <c r="Q47" s="12"/>
@@ -3951,9 +3998,7 @@
       <c r="L48" s="17">
         <v>12</v>
       </c>
-      <c r="M48" s="18">
-        <v>1</v>
-      </c>
+      <c r="M48" s="18"/>
       <c r="N48" s="18">
         <v>2</v>
       </c>
@@ -3997,9 +4042,7 @@
       <c r="L49" s="17">
         <v>12</v>
       </c>
-      <c r="M49" s="18">
-        <v>1</v>
-      </c>
+      <c r="M49" s="18"/>
       <c r="N49" s="18">
         <v>2</v>
       </c>
@@ -4043,9 +4086,7 @@
       <c r="L50" s="17">
         <v>12</v>
       </c>
-      <c r="M50" s="18">
-        <v>1</v>
-      </c>
+      <c r="M50" s="18"/>
       <c r="N50" s="18">
         <v>1</v>
       </c>
@@ -4085,9 +4126,7 @@
       <c r="L51" s="17">
         <v>12</v>
       </c>
-      <c r="M51" s="18">
-        <v>1</v>
-      </c>
+      <c r="M51" s="18"/>
       <c r="N51" s="18">
         <v>1</v>
       </c>
@@ -4131,9 +4170,7 @@
       <c r="L52" s="17">
         <v>12</v>
       </c>
-      <c r="M52" s="18">
-        <v>1</v>
-      </c>
+      <c r="M52" s="18"/>
       <c r="N52" s="18">
         <v>1</v>
       </c>
@@ -4177,9 +4214,7 @@
       <c r="L53" s="17">
         <v>12</v>
       </c>
-      <c r="M53" s="18">
-        <v>1</v>
-      </c>
+      <c r="M53" s="18"/>
       <c r="N53" s="18">
         <v>1</v>
       </c>
@@ -4223,9 +4258,7 @@
       <c r="L54" s="17">
         <v>12</v>
       </c>
-      <c r="M54" s="18">
-        <v>1</v>
-      </c>
+      <c r="M54" s="18"/>
       <c r="N54" s="18">
         <v>1</v>
       </c>
@@ -4269,9 +4302,7 @@
       <c r="L55" s="17">
         <v>12</v>
       </c>
-      <c r="M55" s="18">
-        <v>1</v>
-      </c>
+      <c r="M55" s="18"/>
       <c r="N55" s="18">
         <v>1</v>
       </c>
@@ -4315,9 +4346,7 @@
       <c r="L56" s="17">
         <v>12</v>
       </c>
-      <c r="M56" s="18">
-        <v>1</v>
-      </c>
+      <c r="M56" s="18"/>
       <c r="N56" s="18">
         <v>1</v>
       </c>
@@ -4399,9 +4428,7 @@
       <c r="L58" s="17">
         <v>12</v>
       </c>
-      <c r="M58" s="18">
-        <v>1</v>
-      </c>
+      <c r="M58" s="18"/>
       <c r="N58" s="18">
         <v>1</v>
       </c>
@@ -4441,9 +4468,7 @@
       <c r="L59" s="17">
         <v>12</v>
       </c>
-      <c r="M59" s="18">
-        <v>1</v>
-      </c>
+      <c r="M59" s="18"/>
       <c r="N59" s="18">
         <v>1</v>
       </c>
@@ -4483,9 +4508,7 @@
       <c r="L60" s="17">
         <v>12</v>
       </c>
-      <c r="M60" s="18">
-        <v>1</v>
-      </c>
+      <c r="M60" s="18"/>
       <c r="N60" s="18">
         <v>1</v>
       </c>
@@ -4497,42 +4520,40 @@
       <c r="Q60" s="12"/>
     </row>
     <row r="61" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="13" t="s">
+      <c r="A61" s="42" t="s">
         <v>370</v>
       </c>
-      <c r="B61" s="14" t="s">
+      <c r="B61" s="43" t="s">
         <v>182</v>
       </c>
-      <c r="C61" s="13" t="s">
+      <c r="C61" s="42" t="s">
         <v>197</v>
       </c>
-      <c r="D61" s="13" t="s">
+      <c r="D61" s="42" t="s">
         <v>198</v>
       </c>
-      <c r="E61" s="13" t="s">
+      <c r="E61" s="42" t="s">
         <v>399</v>
       </c>
-      <c r="F61" s="13" t="s">
+      <c r="F61" s="42" t="s">
         <v>400</v>
       </c>
-      <c r="G61" s="13"/>
-      <c r="H61" s="13"/>
-      <c r="I61" s="13" t="s">
+      <c r="G61" s="42"/>
+      <c r="H61" s="42"/>
+      <c r="I61" s="42" t="s">
         <v>401</v>
       </c>
-      <c r="J61" s="13" t="s">
+      <c r="J61" s="42" t="s">
         <v>402</v>
       </c>
-      <c r="K61" s="33">
+      <c r="K61" s="44">
         <v>1</v>
       </c>
-      <c r="L61" s="17">
-        <v>12</v>
-      </c>
-      <c r="M61" s="18">
-        <v>1</v>
-      </c>
-      <c r="N61" s="18">
+      <c r="L61" s="45">
+        <v>12</v>
+      </c>
+      <c r="M61" s="46"/>
+      <c r="N61" s="46">
         <v>1</v>
       </c>
       <c r="O61" s="11">
@@ -4543,45 +4564,43 @@
       <c r="Q61" s="12"/>
     </row>
     <row r="62" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="13" t="s">
+      <c r="A62" s="47" t="s">
         <v>370</v>
       </c>
-      <c r="B62" s="14" t="s">
+      <c r="B62" s="48" t="s">
         <v>182</v>
       </c>
-      <c r="C62" s="13" t="s">
+      <c r="C62" s="47" t="s">
         <v>200</v>
       </c>
-      <c r="D62" s="13" t="s">
+      <c r="D62" s="47" t="s">
         <v>201</v>
       </c>
-      <c r="E62" s="13" t="s">
+      <c r="E62" s="47" t="s">
         <v>403</v>
       </c>
-      <c r="F62" s="13" t="s">
+      <c r="F62" s="47" t="s">
         <v>404</v>
       </c>
-      <c r="G62" s="13"/>
-      <c r="H62" s="13"/>
-      <c r="I62" s="13" t="s">
+      <c r="G62" s="47"/>
+      <c r="H62" s="47"/>
+      <c r="I62" s="47" t="s">
         <v>405</v>
       </c>
-      <c r="J62" s="13" t="s">
+      <c r="J62" s="47" t="s">
         <v>406</v>
       </c>
-      <c r="K62" s="21">
+      <c r="K62" s="49">
         <v>0.95</v>
       </c>
-      <c r="L62" s="17">
-        <v>12</v>
-      </c>
-      <c r="M62" s="18">
+      <c r="L62" s="50">
+        <v>12</v>
+      </c>
+      <c r="M62" s="51"/>
+      <c r="N62" s="51">
         <v>1</v>
       </c>
-      <c r="N62" s="18">
-        <v>1</v>
-      </c>
-      <c r="O62" s="11">
+      <c r="O62" s="52">
         <f t="shared" si="1"/>
         <v>0.95</v>
       </c>
@@ -4589,61 +4608,61 @@
       <c r="Q62" s="12"/>
     </row>
     <row r="63" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="34"/>
-      <c r="B63" s="34"/>
-      <c r="C63" s="34"/>
-      <c r="D63" s="34"/>
-      <c r="E63" s="34"/>
-      <c r="F63" s="34"/>
-      <c r="G63" s="34"/>
-      <c r="H63" s="34"/>
-      <c r="I63" s="34"/>
-      <c r="J63" s="34"/>
-      <c r="K63" s="11"/>
-      <c r="L63" s="35"/>
-      <c r="M63" s="12"/>
-      <c r="N63" s="12"/>
-      <c r="O63" s="36"/>
+      <c r="A63" s="48" t="s">
+        <v>227</v>
+      </c>
+      <c r="B63" s="48" t="s">
+        <v>409</v>
+      </c>
+      <c r="C63" s="48" t="s">
+        <v>408</v>
+      </c>
+      <c r="D63" s="48" t="s">
+        <v>410</v>
+      </c>
+      <c r="E63" s="48"/>
+      <c r="F63" s="48"/>
+      <c r="G63" s="48"/>
+      <c r="H63" s="48"/>
+      <c r="I63" s="48"/>
+      <c r="J63" s="48"/>
+      <c r="K63" s="55">
+        <v>1.5</v>
+      </c>
+      <c r="L63" s="56">
+        <v>12</v>
+      </c>
+      <c r="M63" s="53">
+        <v>3.35</v>
+      </c>
+      <c r="N63" s="53">
+        <v>6.67</v>
+      </c>
+      <c r="O63" s="54">
+        <f t="shared" si="1"/>
+        <v>10.004999999999999</v>
+      </c>
       <c r="P63" s="12"/>
       <c r="Q63" s="30"/>
     </row>
     <row r="64" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="34"/>
-      <c r="B64" s="34"/>
-      <c r="C64" s="34"/>
-      <c r="D64" s="34"/>
-      <c r="E64" s="34"/>
-      <c r="F64" s="34"/>
-      <c r="G64" s="34"/>
-      <c r="H64" s="34"/>
-      <c r="I64" s="34"/>
-      <c r="J64" s="34"/>
+      <c r="A64" s="33"/>
+      <c r="B64" s="33"/>
+      <c r="C64" s="33"/>
+      <c r="D64" s="33"/>
+      <c r="E64" s="33"/>
+      <c r="F64" s="33"/>
+      <c r="G64" s="33"/>
+      <c r="H64" s="33"/>
+      <c r="I64" s="33"/>
+      <c r="J64" s="33"/>
       <c r="K64" s="11"/>
-      <c r="L64" s="35"/>
+      <c r="L64" s="34"/>
       <c r="M64" s="12"/>
       <c r="N64" s="12"/>
-      <c r="O64" s="36"/>
+      <c r="O64" s="35"/>
       <c r="P64" s="12"/>
-      <c r="Q64" s="30"/>
-    </row>
-    <row r="65" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="34"/>
-      <c r="B65" s="34"/>
-      <c r="C65" s="34"/>
-      <c r="D65" s="34"/>
-      <c r="E65" s="34"/>
-      <c r="F65" s="34"/>
-      <c r="G65" s="34"/>
-      <c r="H65" s="34"/>
-      <c r="I65" s="34"/>
-      <c r="J65" s="34"/>
-      <c r="K65" s="11"/>
-      <c r="L65" s="35"/>
-      <c r="M65" s="12"/>
-      <c r="N65" s="12"/>
-      <c r="O65" s="36"/>
-      <c r="P65" s="12"/>
-      <c r="Q65" s="29"/>
+      <c r="Q64" s="29"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="M1:N1048576">
@@ -4667,7 +4686,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D63"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.5" style="3" bestFit="1" customWidth="1"/>
@@ -5503,45 +5522,59 @@
       </c>
     </row>
     <row r="60" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="2" t="s">
+      <c r="A60" s="57" t="s">
         <v>182</v>
       </c>
-      <c r="B60" s="2" t="s">
+      <c r="B60" s="57" t="s">
         <v>194</v>
       </c>
-      <c r="C60" s="2" t="s">
+      <c r="C60" s="57" t="s">
         <v>195</v>
       </c>
-      <c r="D60" s="2" t="s">
+      <c r="D60" s="57" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="2" t="s">
+      <c r="A61" s="58" t="s">
         <v>182</v>
       </c>
-      <c r="B61" s="2" t="s">
+      <c r="B61" s="58" t="s">
         <v>197</v>
       </c>
-      <c r="C61" s="2" t="s">
+      <c r="C61" s="58" t="s">
         <v>198</v>
       </c>
-      <c r="D61" s="2" t="s">
+      <c r="D61" s="58" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="2" t="s">
+      <c r="A62" s="58" t="s">
         <v>182</v>
       </c>
-      <c r="B62" s="2" t="s">
+      <c r="B62" s="58" t="s">
         <v>200</v>
       </c>
-      <c r="C62" s="2" t="s">
+      <c r="C62" s="58" t="s">
         <v>201</v>
       </c>
-      <c r="D62" s="2" t="s">
+      <c r="D62" s="58" t="s">
         <v>202</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" s="59" t="s">
+        <v>409</v>
+      </c>
+      <c r="B63" s="59" t="s">
+        <v>408</v>
+      </c>
+      <c r="C63" s="59" t="s">
+        <v>410</v>
+      </c>
+      <c r="D63" s="59" t="s">
+        <v>411</v>
       </c>
     </row>
   </sheetData>

</xml_diff>